<commit_message>
fix: match import schools by level
</commit_message>
<xml_diff>
--- a/public/templates/shs_teacher_import_template.xlsx
+++ b/public/templates/shs_teacher_import_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="77">
   <si>
     <r>
       <rPr>
@@ -169,15 +169,18 @@
     <t>Agripino Alvarez Elementary School</t>
   </si>
   <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>STEM</t>
+  </si>
+  <si>
+    <t>Cambogui-ot National High School</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
-    <t>STEM</t>
-  </si>
-  <si>
-    <t>Cambogui-ot National High School</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
@@ -187,15 +190,18 @@
     <t>Banag Elementary School</t>
   </si>
   <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>ABM</t>
+  </si>
+  <si>
+    <t>Camindangan National High School</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
-    <t>ABM</t>
-  </si>
-  <si>
-    <t>Camindangan National High School</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -205,61 +211,55 @@
     <t>Barangay V Elementary School</t>
   </si>
   <si>
+    <t>HUMSS</t>
+  </si>
+  <si>
+    <t>Cayhagan National High School</t>
+  </si>
+  <si>
     <t>3</t>
   </si>
   <si>
-    <t>HUMSS</t>
-  </si>
-  <si>
-    <t>Cayhagan National High School</t>
-  </si>
-  <si>
     <t>9</t>
   </si>
   <si>
     <t>Barasbarasan Elementary School</t>
   </si>
   <si>
+    <t>GAS</t>
+  </si>
+  <si>
+    <t>Dung-i Integrated School</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
-    <t>GAS</t>
-  </si>
-  <si>
-    <t>Dung-i Integrated School</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
     <t>Bawog Elementary School</t>
   </si>
   <si>
+    <t>TVL-HE</t>
+  </si>
+  <si>
+    <t>Dungga Integrated School</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
-    <t>TVL-HE</t>
-  </si>
-  <si>
-    <t>Dungga Integrated School</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
     <t>Binotusan Elementary School</t>
   </si>
   <si>
+    <t>TVL-ICT</t>
+  </si>
+  <si>
+    <t>Gil Montilla National High School</t>
+  </si>
+  <si>
     <t>6</t>
-  </si>
-  <si>
-    <t>TVL-ICT</t>
-  </si>
-  <si>
-    <t>Gil Montilla National High School</t>
-  </si>
-  <si>
-    <t>12</t>
   </si>
   <si>
     <t>Binulig Elementary School</t>
@@ -910,12 +910,18 @@
     <row r="100" spans="3:5" x14ac:dyDescent="0.25"/>
     <row r="101" spans="3:5" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select School" prompt="Choose from the list" sqref="C10:C101">
       <formula1>Dropdowns!$A$1:$A$45</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select School" prompt="Choose from the list" sqref="C2:C101">
       <formula1>Dropdowns!$A$1:$A$45</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="D10:D101">
+      <formula1>Dropdowns!$B$1:$B$2</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="D2:D101">
+      <formula1>Dropdowns!$B$1:$B$2</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Track/Strand" prompt="Choose from the list" sqref="E10:E101">
       <formula1>Dropdowns!$C$1:$C$10</formula1>
@@ -951,140 +957,125 @@
         <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
-        <v>25</v>
-      </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
-        <v>30</v>
-      </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" t="s">
         <v>36</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
         <v>38</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
       <c r="C7" t="s">
         <v>41</v>
       </c>
@@ -1099,9 +1090,6 @@
       <c r="A8" t="s">
         <v>43</v>
       </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
       <c r="C8" t="s">
         <v>44</v>
       </c>
@@ -1116,9 +1104,6 @@
       <c r="A9" t="s">
         <v>46</v>
       </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
       <c r="C9" t="s">
         <v>47</v>
       </c>
@@ -1133,9 +1118,6 @@
       <c r="A10" t="s">
         <v>49</v>
       </c>
-      <c r="B10" t="s">
-        <v>29</v>
-      </c>
       <c r="C10" t="s">
         <v>50</v>
       </c>
@@ -1150,9 +1132,6 @@
       <c r="A11" t="s">
         <v>52</v>
       </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
       <c r="D11" t="s">
         <v>52</v>
       </c>
@@ -1164,9 +1143,6 @@
       <c r="A12" t="s">
         <v>54</v>
       </c>
-      <c r="B12" t="s">
-        <v>39</v>
-      </c>
       <c r="D12" t="s">
         <v>54</v>
       </c>
@@ -1198,7 +1174,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
         <v>60</v>
@@ -1255,7 +1231,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D21" t="s">
         <v>69</v>
@@ -1271,7 +1247,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
         <v>71</v>
@@ -1279,7 +1255,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D24" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
fix: require deped email in teacher imports
</commit_message>
<xml_diff>
--- a/public/templates/shs_teacher_import_template.xlsx
+++ b/public/templates/shs_teacher_import_template.xlsx
@@ -153,7 +153,7 @@
         <color rgb="FFFFFFFF"/>
         <sz val="11"/>
       </rPr>
-      <t xml:space="preserve">Email
+      <t xml:space="preserve">Email/DepEd Email
 </t>
     </r>
     <r>
@@ -162,7 +162,7 @@
         <color rgb="FFFFFFFF"/>
         <sz val="9"/>
       </rPr>
-      <t>(optional)</t>
+      <t>(required)</t>
     </r>
   </si>
   <si>

</xml_diff>